<commit_message>
fix: resolve vocab UI issues, save button, and lesson state sync
</commit_message>
<xml_diff>
--- a/file_vocab/thang trong tien trung.xlsx
+++ b/file_vocab/thang trong tien trung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>一 月</t>
   </si>
@@ -60,6 +60,30 @@
   </si>
   <si>
     <t>十 二 月</t>
+  </si>
+  <si>
+    <t>星期 一</t>
+  </si>
+  <si>
+    <t>星期 二</t>
+  </si>
+  <si>
+    <t>星期 三</t>
+  </si>
+  <si>
+    <t>星期 四</t>
+  </si>
+  <si>
+    <t>星期 五</t>
+  </si>
+  <si>
+    <t>星期 六</t>
+  </si>
+  <si>
+    <t>星期 七</t>
+  </si>
+  <si>
+    <t>星期日， 星期天</t>
   </si>
 </sst>
 </file>
@@ -377,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -440,6 +464,46 @@
         <v>11</v>
       </c>
     </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>